<commit_message>
docs(v2): extension roadmap — efficacité du modèle (feuille Excel)
Ajoute la feuille « 8. Efficacité modèle » au classeur de roadmap V2 : diagnostic
chiffré de l'existant (Ministral-3-8B QLoRA r=16, corpus 10k AUTO-généré par le
modèle lui-même, GGUF Q4_K_M ~1 min/réponse) et backlog des leviers d'efficacité
(F1-F12) regroupés en 3 phases :
- mesure d'abord (éval étendue + bench latence + juge GLM-5.2) ;
- corpus distillé depuis un VRAI maître (GLM-5.2 / Qwen2.5-72B) + refus 17 -> 300 ;
- entraînement piloté par l'éval + DPO ; quantization imatrix ; serving llama.cpp
  (flash-attn, KV q8, cache de préfixe) ; RAG embeddings forts + reranking ;
  boucle juge -> curation -> ré-entraînement.
Plus une combinaison recommandée (qualité × latence × souveraineté).
</commit_message>
<xml_diff>
--- a/docs/OpenCacao_V2_Roadmap_Agile.xlsx
+++ b/docs/OpenCacao_V2_Roadmap_Agile.xlsx
@@ -15,6 +15,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="5. Rétro-planning" sheetId="6" state="visible" r:id="rId6"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="6. Gantt" sheetId="7" state="visible" r:id="rId7"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="7. Risques" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="8. Efficacité modèle" sheetId="9" state="visible" r:id="rId9"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -24,7 +25,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="21">
+  <fonts count="22">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -122,8 +123,12 @@
     <font>
       <sz val="9"/>
     </font>
+    <font>
+      <color rgb="003F3F3F"/>
+      <sz val="8"/>
+    </font>
   </fonts>
-  <fills count="20">
+  <fills count="21">
     <fill>
       <patternFill/>
     </fill>
@@ -220,6 +225,11 @@
         <fgColor rgb="00FFE0B2"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00B8410A"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -247,7 +257,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="74">
+  <cellXfs count="81">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -449,6 +459,27 @@
     </xf>
     <xf numFmtId="0" fontId="11" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="20" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="9" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1" indent="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -884,7 +915,7 @@
     <row r="16" ht="26" customHeight="1">
       <c r="A16" s="3" t="inlineStr">
         <is>
-          <t>Assistant 100 % conversationnel — mémoire &amp; sessions persistantes</t>
+          <t>Assistant conversationnel — mémoire, sessions &amp; efficacité du modèle</t>
         </is>
       </c>
     </row>
@@ -4745,4 +4776,550 @@
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F27"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="7" customWidth="1" min="1" max="1"/>
+    <col width="24" customWidth="1" min="2" max="2"/>
+    <col width="60" customWidth="1" min="3" max="3"/>
+    <col width="11" customWidth="1" min="4" max="4"/>
+    <col width="8" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="34" customHeight="1">
+      <c r="A1" s="9" t="inlineStr">
+        <is>
+          <t>Extension V2 — Efficacité du modèle</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="20" customHeight="1">
+      <c r="A2" s="10" t="inlineStr">
+        <is>
+          <t>Qualité + latence : entraînement RunPod (GPU 24 Go) → service K3s CX53 (CPU, GGUF llama.cpp)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="24" customHeight="1">
+      <c r="A4" s="74" t="inlineStr">
+        <is>
+          <t>Modèle</t>
+        </is>
+      </c>
+      <c r="B4" s="75" t="inlineStr">
+        <is>
+          <t>Ministral-3-8B-Instruct-2512 · QLoRA r=16/α=32 NF4 · 1 epoch · GGUF Q4_K_M (~5 Go).</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="24" customHeight="1">
+      <c r="A5" s="74" t="inlineStr">
+        <is>
+          <t>Service</t>
+        </is>
+      </c>
+      <c r="B5" s="76" t="inlineStr">
+        <is>
+          <t>llama.cpp CPU sur CX53 (16 vCPU/32 Go), -c 4096, -t 12 ≈ 10-15 tok/s ≈ 1 min/réponse.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="24" customHeight="1">
+      <c r="A6" s="74" t="inlineStr">
+        <is>
+          <t>Corpus</t>
+        </is>
+      </c>
+      <c r="B6" s="75" t="inlineStr">
+        <is>
+          <t>10 000 paires AUTO-générées par Ministral-8B lui-même (pas un maître) + 17 refus + 20 amorce.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="24" customHeight="1">
+      <c r="A7" s="77" t="inlineStr">
+        <is>
+          <t>Point faible #1</t>
+        </is>
+      </c>
+      <c r="B7" s="76" t="inlineStr">
+        <is>
+          <t>Auto-distillation : le fine-tune ne peut PAS dépasser le modèle de base. Plafond de qualité bridé.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="24" customHeight="1">
+      <c r="A8" s="77" t="inlineStr">
+        <is>
+          <t>Point faible #2</t>
+        </is>
+      </c>
+      <c r="B8" s="75" t="inlineStr">
+        <is>
+          <t>Seulement 17 exemples de refus ; éval = 20 cas ; pas de validation pilotant le choix de checkpoint.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="24" customHeight="1">
+      <c r="A9" s="77" t="inlineStr">
+        <is>
+          <t>Point faible #3</t>
+        </is>
+      </c>
+      <c r="B9" s="76" t="inlineStr">
+        <is>
+          <t>Latence ~1 min/réponse (UX) ; quantization Q4_K_M sans imatrix ; pas de cache de préfixe ni KV-quant.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="24" customHeight="1">
+      <c r="A10" s="74" t="inlineStr">
+        <is>
+          <t>Atouts en place</t>
+        </is>
+      </c>
+      <c r="B10" s="75" t="inlineStr">
+        <is>
+          <t>Pipeline RunPod complet, maître souverain dispo (GLM-5.2 / Qwen2.5-72B), RAG actif, journal 👍/👎.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="26" customHeight="1">
+      <c r="A12" s="19" t="inlineStr">
+        <is>
+          <t>ID</t>
+        </is>
+      </c>
+      <c r="B12" s="19" t="inlineStr">
+        <is>
+          <t>Lot</t>
+        </is>
+      </c>
+      <c r="C12" s="19" t="inlineStr">
+        <is>
+          <t>Levier (user story)</t>
+        </is>
+      </c>
+      <c r="D12" s="19" t="inlineStr">
+        <is>
+          <t>Priorité</t>
+        </is>
+      </c>
+      <c r="E12" s="19" t="inlineStr">
+        <is>
+          <t>SP</t>
+        </is>
+      </c>
+      <c r="F12" s="19" t="inlineStr">
+        <is>
+          <t>Phase</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="30" customHeight="1">
+      <c r="A13" s="45" t="inlineStr">
+        <is>
+          <t>F1</t>
+        </is>
+      </c>
+      <c r="B13" s="78" t="inlineStr">
+        <is>
+          <t>1 Mesure</t>
+        </is>
+      </c>
+      <c r="C13" s="23" t="inlineStr">
+        <is>
+          <t>Étendre l'éval (20 → ~150 cas, multi-tours/refus) + bench de latence + juge GLM-5.2 intégré.</t>
+        </is>
+      </c>
+      <c r="D13" s="24" t="inlineStr">
+        <is>
+          <t>Must</t>
+        </is>
+      </c>
+      <c r="E13" s="21" t="n">
+        <v>5</v>
+      </c>
+      <c r="F13" s="27" t="inlineStr">
+        <is>
+          <t>Ext-S1</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="30" customHeight="1">
+      <c r="A14" s="45" t="inlineStr">
+        <is>
+          <t>F2</t>
+        </is>
+      </c>
+      <c r="B14" s="78" t="inlineStr">
+        <is>
+          <t>2 Corpus maître</t>
+        </is>
+      </c>
+      <c r="C14" s="23" t="inlineStr">
+        <is>
+          <t>Distiller depuis un VRAI maître (GLM-5.2 ceiling + Qwen2.5-72B-AWQ souverain) au lieu de l'auto-génération.</t>
+        </is>
+      </c>
+      <c r="D14" s="24" t="inlineStr">
+        <is>
+          <t>Must</t>
+        </is>
+      </c>
+      <c r="E14" s="21" t="n">
+        <v>8</v>
+      </c>
+      <c r="F14" s="27" t="inlineStr">
+        <is>
+          <t>Ext-S1</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="30" customHeight="1">
+      <c r="A15" s="45" t="inlineStr">
+        <is>
+          <t>F3</t>
+        </is>
+      </c>
+      <c r="B15" s="78" t="inlineStr">
+        <is>
+          <t>2 Corpus maître</t>
+        </is>
+      </c>
+      <c r="C15" s="23" t="inlineStr">
+        <is>
+          <t>Élargir les refus 17 → ~300 (évasion dose multi-tours, médical, image, hors-filière).</t>
+        </is>
+      </c>
+      <c r="D15" s="24" t="inlineStr">
+        <is>
+          <t>Must</t>
+        </is>
+      </c>
+      <c r="E15" s="21" t="n">
+        <v>5</v>
+      </c>
+      <c r="F15" s="27" t="inlineStr">
+        <is>
+          <t>Ext-S1</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="30" customHeight="1">
+      <c r="A16" s="45" t="inlineStr">
+        <is>
+          <t>F4</t>
+        </is>
+      </c>
+      <c r="B16" s="78" t="inlineStr">
+        <is>
+          <t>3 Entraînement</t>
+        </is>
+      </c>
+      <c r="C16" s="23" t="inlineStr">
+        <is>
+          <t>Recette pilotée par l'éval : sweep epochs (1/2/3) × rang LoRA (16/32/64) × lr ; meilleur checkpoint ; max_seq 1024→1536.</t>
+        </is>
+      </c>
+      <c r="D16" s="28" t="inlineStr">
+        <is>
+          <t>Should</t>
+        </is>
+      </c>
+      <c r="E16" s="21" t="n">
+        <v>5</v>
+      </c>
+      <c r="F16" s="29" t="inlineStr">
+        <is>
+          <t>Ext-S2</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="30" customHeight="1">
+      <c r="A17" s="45" t="inlineStr">
+        <is>
+          <t>F5</t>
+        </is>
+      </c>
+      <c r="B17" s="78" t="inlineStr">
+        <is>
+          <t>4 Alignement</t>
+        </is>
+      </c>
+      <c r="C17" s="23" t="inlineStr">
+        <is>
+          <t>DPO/ORPO sur ~1-2k paires de préférence (concision « SMS », citation de source, refus nets).</t>
+        </is>
+      </c>
+      <c r="D17" s="28" t="inlineStr">
+        <is>
+          <t>Should</t>
+        </is>
+      </c>
+      <c r="E17" s="21" t="n">
+        <v>8</v>
+      </c>
+      <c r="F17" s="29" t="inlineStr">
+        <is>
+          <t>Ext-S2</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="30" customHeight="1">
+      <c r="A18" s="45" t="inlineStr">
+        <is>
+          <t>F11</t>
+        </is>
+      </c>
+      <c r="B18" s="78" t="inlineStr">
+        <is>
+          <t>7 Boucle</t>
+        </is>
+      </c>
+      <c r="C18" s="23" t="inlineStr">
+        <is>
+          <t>Juge GLM-5.2 sur le journal de prod (👍/👎) → corpus curé → ré-entraînement périodique.</t>
+        </is>
+      </c>
+      <c r="D18" s="24" t="inlineStr">
+        <is>
+          <t>Must</t>
+        </is>
+      </c>
+      <c r="E18" s="21" t="n">
+        <v>5</v>
+      </c>
+      <c r="F18" s="29" t="inlineStr">
+        <is>
+          <t>Ext-S2</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="30" customHeight="1">
+      <c r="A19" s="45" t="inlineStr">
+        <is>
+          <t>F6</t>
+        </is>
+      </c>
+      <c r="B19" s="78" t="inlineStr">
+        <is>
+          <t>5 Quantization</t>
+        </is>
+      </c>
+      <c r="C19" s="23" t="inlineStr">
+        <is>
+          <t>Quantization imatrix (calibration sur le corpus domaine) → Q4_K_M-imatrix ; comparer Q4_K_M-imatrix vs Q5_K_M.</t>
+        </is>
+      </c>
+      <c r="D19" s="28" t="inlineStr">
+        <is>
+          <t>Should</t>
+        </is>
+      </c>
+      <c r="E19" s="21" t="n">
+        <v>3</v>
+      </c>
+      <c r="F19" s="30" t="inlineStr">
+        <is>
+          <t>Ext-S3</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="30" customHeight="1">
+      <c r="A20" s="45" t="inlineStr">
+        <is>
+          <t>F7</t>
+        </is>
+      </c>
+      <c r="B20" s="78" t="inlineStr">
+        <is>
+          <t>5 Serving</t>
+        </is>
+      </c>
+      <c r="C20" s="23" t="inlineStr">
+        <is>
+          <t>llama.cpp : flash-attn, KV-cache q8, cache de préfixe (prompt système figé), threads, max_tokens 512→384.</t>
+        </is>
+      </c>
+      <c r="D20" s="28" t="inlineStr">
+        <is>
+          <t>Should</t>
+        </is>
+      </c>
+      <c r="E20" s="21" t="n">
+        <v>5</v>
+      </c>
+      <c r="F20" s="30" t="inlineStr">
+        <is>
+          <t>Ext-S3</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="30" customHeight="1">
+      <c r="A21" s="45" t="inlineStr">
+        <is>
+          <t>F8</t>
+        </is>
+      </c>
+      <c r="B21" s="78" t="inlineStr">
+        <is>
+          <t>5 Serving</t>
+        </is>
+      </c>
+      <c r="C21" s="23" t="inlineStr">
+        <is>
+          <t>Décodage spéculatif (petit modèle brouillon) pour accélérer la génération sur CPU.</t>
+        </is>
+      </c>
+      <c r="D21" s="31" t="inlineStr">
+        <is>
+          <t>Could</t>
+        </is>
+      </c>
+      <c r="E21" s="21" t="n">
+        <v>5</v>
+      </c>
+      <c r="F21" s="30" t="inlineStr">
+        <is>
+          <t>Ext-S3</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="30" customHeight="1">
+      <c r="A22" s="45" t="inlineStr">
+        <is>
+          <t>F9</t>
+        </is>
+      </c>
+      <c r="B22" s="78" t="inlineStr">
+        <is>
+          <t>6 RAG</t>
+        </is>
+      </c>
+      <c r="C22" s="23" t="inlineStr">
+        <is>
+          <t>Embeddings plus forts (multilingual-e5 / BGE-M3) + top_k 8 → reranking → 3 ; calibrer le seuil.</t>
+        </is>
+      </c>
+      <c r="D22" s="28" t="inlineStr">
+        <is>
+          <t>Should</t>
+        </is>
+      </c>
+      <c r="E22" s="21" t="n">
+        <v>5</v>
+      </c>
+      <c r="F22" s="30" t="inlineStr">
+        <is>
+          <t>Ext-S3</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="30" customHeight="1">
+      <c r="A23" s="45" t="inlineStr">
+        <is>
+          <t>F10</t>
+        </is>
+      </c>
+      <c r="B23" s="78" t="inlineStr">
+        <is>
+          <t>6 RAG</t>
+        </is>
+      </c>
+      <c r="C23" s="23" t="inlineStr">
+        <is>
+          <t>Récupération hybride BM25 + dense (recall sur noms de maladies/variétés).</t>
+        </is>
+      </c>
+      <c r="D23" s="31" t="inlineStr">
+        <is>
+          <t>Could</t>
+        </is>
+      </c>
+      <c r="E23" s="21" t="n">
+        <v>3</v>
+      </c>
+      <c r="F23" s="30" t="inlineStr">
+        <is>
+          <t>Ext-S3</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="30" customHeight="1">
+      <c r="A24" s="45" t="inlineStr">
+        <is>
+          <t>F12</t>
+        </is>
+      </c>
+      <c r="B24" s="78" t="inlineStr">
+        <is>
+          <t>1 Mesure</t>
+        </is>
+      </c>
+      <c r="C24" s="23" t="inlineStr">
+        <is>
+          <t>Harnais A/B (qualité + latence) comparant les versions de modèle, choix de la version à déployer.</t>
+        </is>
+      </c>
+      <c r="D24" s="31" t="inlineStr">
+        <is>
+          <t>Could</t>
+        </is>
+      </c>
+      <c r="E24" s="21" t="n">
+        <v>3</v>
+      </c>
+      <c r="F24" s="30" t="inlineStr">
+        <is>
+          <t>Ext-S3</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="22" customHeight="1">
+      <c r="A26" s="79" t="inlineStr">
+        <is>
+          <t>Combinaison recommandée (qualité × latence × souveraineté)</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="92" customHeight="1">
+      <c r="A27" s="80" t="inlineStr">
+        <is>
+          <t>Maître : GLM-5.2 (plafond de qualité) sur un sous-ensemble curé + Qwen2.5-72B-AWQ (volume souverain) → corpus ~10-12k + 300 refus.  Entraînement : LoRA r=32, 2 epochs, choix de checkpoint par l'éval, puis DPO sur préférences.  Quantization : Q4_K_M avec imatrix domaine.  Service : flash-attn + KV q8 + cache de préfixe + max_tokens 384 (threads calibrés).  RAG : embeddings multilingual-e5 + reranking.  Boucle : juge GLM-5.2 sur le journal → curation → ré-entraînement mensuel.  Toute combinaison est jugée sur l'éval étendu (F1) : on ne déploie une version que si garde-fous = 100 % ET qualité ≥ baseline ET latence acceptable.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="18">
+    <mergeCell ref="B4:F4"/>
+    <mergeCell ref="A2:F2"/>
+    <mergeCell ref="A8"/>
+    <mergeCell ref="A6"/>
+    <mergeCell ref="B7:F7"/>
+    <mergeCell ref="B6:F6"/>
+    <mergeCell ref="A4"/>
+    <mergeCell ref="A9"/>
+    <mergeCell ref="B10:F10"/>
+    <mergeCell ref="A1:F1"/>
+    <mergeCell ref="A7"/>
+    <mergeCell ref="B5:F5"/>
+    <mergeCell ref="A27:F27"/>
+    <mergeCell ref="A10"/>
+    <mergeCell ref="B8:F8"/>
+    <mergeCell ref="A26:F26"/>
+    <mergeCell ref="B9:F9"/>
+    <mergeCell ref="A5"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
docs(backlog): F13 réponses multilingues (EN) — enum langue + prompt EN + cache/RAG par langue
Retrieval cross-lingue déjà acquis via Qwen3-4B (question EN -> fiche FR
retrouvée en prod). Reste l'enum Langue (DTO 'fr' uniquement), le prompt
système EN et la clé cache/RAG par langue. Could, Ext-S3.
</commit_message>
<xml_diff>
--- a/docs/OpenCacao_V2_Roadmap_Agile.xlsx
+++ b/docs/OpenCacao_V2_Roadmap_Agile.xlsx
@@ -4784,7 +4784,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F27"/>
+  <dimension ref="A1:F28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -5285,15 +5285,45 @@
         </is>
       </c>
     </row>
-    <row r="26" ht="22" customHeight="1">
-      <c r="A26" s="79" t="inlineStr">
+    <row r="25" ht="30" customHeight="1">
+      <c r="A25" s="45" t="inlineStr">
+        <is>
+          <t>F13</t>
+        </is>
+      </c>
+      <c r="B25" s="78" t="inlineStr">
+        <is>
+          <t>8 Multilingue</t>
+        </is>
+      </c>
+      <c r="C25" s="23" t="inlineStr">
+        <is>
+          <t>Réponses multilingues (EN) : élargir l'enum Langue (DTO n'accepte que 'fr') + prompt système EN + clé cache/RAG par langue. Retrieval cross-lingue déjà acquis via Qwen3-4B (question EN → fiche FR retrouvée).</t>
+        </is>
+      </c>
+      <c r="D25" s="31" t="inlineStr">
+        <is>
+          <t>Could</t>
+        </is>
+      </c>
+      <c r="E25" s="21" t="n">
+        <v>5</v>
+      </c>
+      <c r="F25" s="30" t="inlineStr">
+        <is>
+          <t>Ext-S3</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="22" customHeight="1">
+      <c r="A27" s="79" t="inlineStr">
         <is>
           <t>Combinaison recommandée (qualité × latence × souveraineté)</t>
         </is>
       </c>
     </row>
-    <row r="27" ht="92" customHeight="1">
-      <c r="A27" s="80" t="inlineStr">
+    <row r="28" ht="92" customHeight="1">
+      <c r="A28" s="80" t="inlineStr">
         <is>
           <t>Maître : GLM-5.2 (plafond de qualité) sur un sous-ensemble curé + Qwen2.5-72B-AWQ (volume souverain) → corpus ~10-12k + 300 refus.  Entraînement : LoRA r=32, 2 epochs, choix de checkpoint par l'éval, puis DPO sur préférences.  Quantization : Q4_K_M avec imatrix domaine.  Service : flash-attn + KV q8 + cache de préfixe + max_tokens 384 (threads calibrés).  RAG : embeddings multilingual-e5 + reranking.  Boucle : juge GLM-5.2 sur le journal → curation → ré-entraînement mensuel.  Toute combinaison est jugée sur l'éval étendu (F1) : on ne déploie une version que si garde-fous = 100 % ET qualité ≥ baseline ET latence acceptable.</t>
         </is>
@@ -5306,6 +5336,7 @@
     <mergeCell ref="A8"/>
     <mergeCell ref="A6"/>
     <mergeCell ref="B7:F7"/>
+    <mergeCell ref="A28:F28"/>
     <mergeCell ref="B6:F6"/>
     <mergeCell ref="A4"/>
     <mergeCell ref="A9"/>
@@ -5316,7 +5347,6 @@
     <mergeCell ref="A27:F27"/>
     <mergeCell ref="A10"/>
     <mergeCell ref="B8:F8"/>
-    <mergeCell ref="A26:F26"/>
     <mergeCell ref="B9:F9"/>
     <mergeCell ref="A5"/>
   </mergeCells>

</xml_diff>